<commit_message>
Chinese supplier quote added to LCSC BOM. Separate Altium generated BOMs added.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/BOM_LCSC.xlsx
+++ b/Deliverables/BOM/BOM_LCSC.xlsx
@@ -1,30 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24430"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\ChrisitanRaun-AnnanasMotor\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ChrisitanRaun-AnnanasMotor\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AE9F3A8-45C5-493B-8453-63A044D0CDAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="282">
   <si>
     <t>S. No.</t>
   </si>
@@ -877,12 +885,24 @@
   <si>
     <t xml:space="preserve">10V 22uF ±10% CASE-A_3216 Tantalum Capacitors ROHS
 </t>
+  </si>
+  <si>
+    <t>Quotation of orignal parts from Chinese supplier</t>
+  </si>
+  <si>
+    <t>out of stock</t>
+  </si>
+  <si>
+    <t>Custom supplier</t>
+  </si>
+  <si>
+    <t>Cstom Supplier</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
@@ -1030,7 +1050,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -1231,15 +1251,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -1371,6 +1382,51 @@
         <color indexed="64"/>
       </right>
       <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
@@ -1383,7 +1439,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="177">
+  <cellXfs count="186">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1494,41 +1550,35 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1627,21 +1677,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1684,7 +1719,7 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1760,63 +1795,63 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1832,9 +1867,6 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1847,7 +1879,7 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1868,19 +1900,7 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="9" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1906,6 +1926,63 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2187,8 +2264,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S63"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AH63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="37" bestFit="1" customWidth="1"/>
@@ -2208,127 +2285,150 @@
     <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="26.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="166" t="s">
+    <row r="1" spans="1:34" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="168" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="167"/>
-      <c r="C1" s="167"/>
-      <c r="D1" s="167"/>
-      <c r="E1" s="167"/>
-      <c r="F1" s="167"/>
-      <c r="G1" s="167"/>
-      <c r="H1" s="167"/>
-      <c r="I1" s="167"/>
-      <c r="J1" s="167"/>
-      <c r="K1" s="167"/>
-      <c r="L1" s="167"/>
-      <c r="M1" s="167"/>
-      <c r="N1" s="167"/>
-      <c r="O1" s="167"/>
-      <c r="P1" s="167"/>
-      <c r="Q1" s="168"/>
-    </row>
-    <row r="2" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="39" t="s">
+      <c r="B1" s="169"/>
+      <c r="C1" s="169"/>
+      <c r="D1" s="169"/>
+      <c r="E1" s="169"/>
+      <c r="F1" s="169"/>
+      <c r="G1" s="169"/>
+      <c r="H1" s="169"/>
+      <c r="I1" s="169"/>
+      <c r="J1" s="169"/>
+      <c r="K1" s="169"/>
+      <c r="L1" s="169"/>
+      <c r="M1" s="169"/>
+      <c r="N1" s="169"/>
+      <c r="O1" s="169"/>
+      <c r="P1" s="169"/>
+      <c r="Q1" s="170"/>
+      <c r="R1" s="168" t="s">
+        <v>49</v>
+      </c>
+      <c r="S1" s="169"/>
+      <c r="T1" s="169"/>
+      <c r="U1" s="169"/>
+      <c r="V1" s="169"/>
+      <c r="W1" s="169"/>
+      <c r="X1" s="169"/>
+      <c r="Y1" s="169"/>
+      <c r="Z1" s="169"/>
+      <c r="AA1" s="169"/>
+      <c r="AB1" s="169"/>
+      <c r="AC1" s="169"/>
+      <c r="AD1" s="169"/>
+      <c r="AE1" s="169"/>
+      <c r="AF1" s="169"/>
+      <c r="AG1" s="169"/>
+      <c r="AH1" s="170"/>
+    </row>
+    <row r="2" spans="1:34" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="49" t="s">
+      <c r="C2" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="49" t="s">
+      <c r="D2" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="49" t="s">
+      <c r="E2" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="49" t="s">
+      <c r="F2" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="49" t="s">
+      <c r="G2" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="49" t="s">
+      <c r="H2" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="49" t="s">
+      <c r="I2" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="49" t="s">
+      <c r="J2" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="49" t="s">
+      <c r="K2" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="49" t="s">
+      <c r="L2" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="49" t="s">
+      <c r="M2" s="47" t="s">
         <v>209</v>
       </c>
-      <c r="N2" s="50" t="s">
+      <c r="N2" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="O2" s="46" t="s">
+      <c r="O2" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="40" t="s">
+      <c r="P2" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="Q2" s="49" t="s">
+      <c r="Q2" s="47" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="47">
+      <c r="R2" s="171" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="3" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="45">
         <v>1</v>
       </c>
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="165" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="102" t="s">
+      <c r="C3" s="95" t="s">
         <v>50</v>
       </c>
-      <c r="D3" s="103" t="s">
+      <c r="D3" s="96" t="s">
         <v>51</v>
       </c>
-      <c r="E3" s="103" t="s">
+      <c r="E3" s="96" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="103" t="s">
+      <c r="F3" s="96" t="s">
         <v>52</v>
       </c>
-      <c r="G3" s="104" t="s">
+      <c r="G3" s="97" t="s">
         <v>53</v>
       </c>
-      <c r="H3" s="70" t="s">
+      <c r="H3" s="68" t="s">
         <v>214</v>
       </c>
-      <c r="I3" s="78" t="s">
+      <c r="I3" s="76" t="s">
         <v>216</v>
       </c>
-      <c r="J3" s="103" t="s">
+      <c r="J3" s="96" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="105">
+      <c r="K3" s="98">
         <v>2100</v>
       </c>
       <c r="L3" s="1">
         <v>5</v>
       </c>
-      <c r="M3" s="81">
+      <c r="M3" s="79">
         <f t="shared" ref="M3:M46" si="0">L3*400</f>
         <v>2000</v>
       </c>
-      <c r="N3" s="74" t="s">
+      <c r="N3" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="51">
+      <c r="O3" s="49">
         <v>6.8199999999999997E-2</v>
       </c>
       <c r="P3" s="3">
@@ -2336,14 +2436,14 @@
         <v>143.22</v>
       </c>
       <c r="Q3" s="4"/>
-      <c r="R3" s="5"/>
+      <c r="R3" s="172"/>
       <c r="S3" s="5"/>
     </row>
-    <row r="4" spans="1:19" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="47">
+    <row r="4" spans="1:34" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="45">
         <v>2</v>
       </c>
-      <c r="B4" s="83"/>
+      <c r="B4" s="167"/>
       <c r="C4" s="23" t="s">
         <v>54</v>
       </c>
@@ -2356,13 +2456,13 @@
       <c r="F4" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="G4" s="72" t="s">
+      <c r="G4" s="70" t="s">
         <v>58</v>
       </c>
-      <c r="H4" s="61" t="s">
+      <c r="H4" s="59" t="s">
         <v>215</v>
       </c>
-      <c r="I4" s="79" t="s">
+      <c r="I4" s="77" t="s">
         <v>216</v>
       </c>
       <c r="J4" s="21" t="s">
@@ -2378,10 +2478,10 @@
         <f t="shared" si="0"/>
         <v>10400</v>
       </c>
-      <c r="N4" s="76" t="s">
+      <c r="N4" s="74" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="52">
+      <c r="O4" s="50">
         <v>4.7000000000000002E-3</v>
       </c>
       <c r="P4" s="9">
@@ -2389,14 +2489,14 @@
         <v>49.35</v>
       </c>
       <c r="Q4" s="10"/>
-      <c r="R4" s="5"/>
+      <c r="R4" s="173"/>
       <c r="S4" s="5"/>
     </row>
-    <row r="5" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="47">
+    <row r="5" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="45">
         <v>3</v>
       </c>
-      <c r="B5" s="83"/>
+      <c r="B5" s="167"/>
       <c r="C5" s="23" t="s">
         <v>59</v>
       </c>
@@ -2412,10 +2512,10 @@
       <c r="G5" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="H5" s="61" t="s">
+      <c r="H5" s="59" t="s">
         <v>218</v>
       </c>
-      <c r="I5" s="62" t="s">
+      <c r="I5" s="60" t="s">
         <v>217</v>
       </c>
       <c r="J5" s="21" t="s">
@@ -2431,10 +2531,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N5" s="76" t="s">
+      <c r="N5" s="74" t="s">
         <v>16</v>
       </c>
-      <c r="O5" s="52">
+      <c r="O5" s="50">
         <v>8.6999999999999994E-2</v>
       </c>
       <c r="P5" s="9">
@@ -2442,14 +2542,14 @@
         <v>36.54</v>
       </c>
       <c r="Q5" s="10"/>
-      <c r="R5" s="5"/>
+      <c r="R5" s="173"/>
       <c r="S5" s="5"/>
     </row>
-    <row r="6" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="47">
+    <row r="6" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="45">
         <v>4</v>
       </c>
-      <c r="B6" s="83"/>
+      <c r="B6" s="167"/>
       <c r="C6" s="23" t="s">
         <v>62</v>
       </c>
@@ -2465,10 +2565,10 @@
       <c r="G6" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="61" t="s">
+      <c r="H6" s="59" t="s">
         <v>262</v>
       </c>
-      <c r="I6" s="62" t="s">
+      <c r="I6" s="60" t="s">
         <v>261</v>
       </c>
       <c r="J6" s="21" t="s">
@@ -2484,25 +2584,25 @@
         <f t="shared" si="0"/>
         <v>1600</v>
       </c>
-      <c r="N6" s="92" t="s">
+      <c r="N6" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="91">
+      <c r="O6" s="84">
         <v>2.3099999999999999E-2</v>
       </c>
-      <c r="P6" s="58">
+      <c r="P6" s="56">
         <f t="shared" si="1"/>
         <v>39.269999999999996</v>
       </c>
       <c r="Q6" s="10"/>
-      <c r="R6" s="5"/>
+      <c r="R6" s="173"/>
       <c r="S6" s="5"/>
     </row>
-    <row r="7" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="47">
+    <row r="7" spans="1:34" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="45">
         <v>5</v>
       </c>
-      <c r="B7" s="83"/>
+      <c r="B7" s="167"/>
       <c r="C7" s="23" t="s">
         <v>66</v>
       </c>
@@ -2518,10 +2618,10 @@
       <c r="G7" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="H7" s="61" t="s">
+      <c r="H7" s="59" t="s">
         <v>263</v>
       </c>
-      <c r="I7" s="62" t="s">
+      <c r="I7" s="60" t="s">
         <v>264</v>
       </c>
       <c r="J7" s="21" t="s">
@@ -2530,32 +2630,32 @@
       <c r="K7" s="19">
         <v>5000</v>
       </c>
-      <c r="L7" s="41">
+      <c r="L7" s="40">
         <v>12</v>
       </c>
       <c r="M7" s="8">
         <f t="shared" si="0"/>
         <v>4800</v>
       </c>
-      <c r="N7" s="92" t="s">
+      <c r="N7" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="63">
+      <c r="O7" s="61">
         <v>2.2000000000000001E-3</v>
       </c>
-      <c r="P7" s="64">
+      <c r="P7" s="62">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="Q7" s="24"/>
-      <c r="R7" s="5"/>
+      <c r="R7" s="173"/>
       <c r="S7" s="5"/>
     </row>
-    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="47">
+    <row r="8" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="45">
         <v>6</v>
       </c>
-      <c r="B8" s="83"/>
+      <c r="B8" s="167"/>
       <c r="C8" s="23" t="s">
         <v>70</v>
       </c>
@@ -2571,10 +2671,10 @@
       <c r="G8" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H8" s="61" t="s">
+      <c r="H8" s="59" t="s">
         <v>265</v>
       </c>
-      <c r="I8" s="62" t="s">
+      <c r="I8" s="60" t="s">
         <v>266</v>
       </c>
       <c r="J8" s="21" t="s">
@@ -2590,10 +2690,10 @@
         <f t="shared" si="0"/>
         <v>1200</v>
       </c>
-      <c r="N8" s="92" t="s">
+      <c r="N8" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="52">
+      <c r="O8" s="50">
         <v>4.1999999999999997E-3</v>
       </c>
       <c r="P8" s="9">
@@ -2601,14 +2701,14 @@
         <v>5.46</v>
       </c>
       <c r="Q8" s="10"/>
-      <c r="R8" s="5"/>
+      <c r="R8" s="173"/>
       <c r="S8" s="5"/>
     </row>
-    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="47">
+    <row r="9" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="45">
         <v>7</v>
       </c>
-      <c r="B9" s="83"/>
+      <c r="B9" s="167"/>
       <c r="C9" s="23" t="s">
         <v>73</v>
       </c>
@@ -2624,10 +2724,10 @@
       <c r="G9" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="H9" s="61" t="s">
+      <c r="H9" s="59" t="s">
         <v>267</v>
       </c>
-      <c r="I9" s="61" t="s">
+      <c r="I9" s="59" t="s">
         <v>268</v>
       </c>
       <c r="J9" s="21" t="s">
@@ -2643,10 +2743,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N9" s="92" t="s">
+      <c r="N9" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="53">
+      <c r="O9" s="51">
         <v>3.0200000000000001E-2</v>
       </c>
       <c r="P9" s="9">
@@ -2654,14 +2754,14 @@
         <v>12.684000000000001</v>
       </c>
       <c r="Q9" s="10"/>
-      <c r="R9" s="5"/>
+      <c r="R9" s="173"/>
       <c r="S9" s="5"/>
     </row>
-    <row r="10" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="47">
+    <row r="10" spans="1:34" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="45">
         <v>8</v>
       </c>
-      <c r="B10" s="83"/>
+      <c r="B10" s="167"/>
       <c r="C10" s="23" t="s">
         <v>77</v>
       </c>
@@ -2674,13 +2774,13 @@
       <c r="F10" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="G10" s="72" t="s">
+      <c r="G10" s="70" t="s">
         <v>219</v>
       </c>
-      <c r="H10" s="61" t="s">
+      <c r="H10" s="59" t="s">
         <v>220</v>
       </c>
-      <c r="I10" s="79" t="s">
+      <c r="I10" s="77" t="s">
         <v>216</v>
       </c>
       <c r="J10" s="21" t="s">
@@ -2696,25 +2796,25 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N10" s="77" t="s">
+      <c r="N10" s="75" t="s">
         <v>16</v>
       </c>
-      <c r="O10" s="56">
+      <c r="O10" s="54">
         <v>5.8500000000000003E-2</v>
       </c>
-      <c r="P10" s="57">
+      <c r="P10" s="55">
         <f t="shared" si="1"/>
         <v>24.57</v>
       </c>
-      <c r="Q10" s="60"/>
-      <c r="R10" s="5"/>
+      <c r="Q10" s="58"/>
+      <c r="R10" s="173"/>
       <c r="S10" s="5"/>
     </row>
-    <row r="11" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="47">
+    <row r="11" spans="1:34" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="45">
         <v>9</v>
       </c>
-      <c r="B11" s="83"/>
+      <c r="B11" s="167"/>
       <c r="C11" s="23" t="s">
         <v>80</v>
       </c>
@@ -2727,13 +2827,13 @@
       <c r="F11" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="G11" s="72" t="s">
+      <c r="G11" s="70" t="s">
         <v>219</v>
       </c>
-      <c r="H11" s="61" t="s">
+      <c r="H11" s="59" t="s">
         <v>221</v>
       </c>
-      <c r="I11" s="79" t="s">
+      <c r="I11" s="77" t="s">
         <v>216</v>
       </c>
       <c r="J11" s="21" t="s">
@@ -2749,25 +2849,25 @@
         <f t="shared" si="0"/>
         <v>800</v>
       </c>
-      <c r="N11" s="77" t="s">
+      <c r="N11" s="75" t="s">
         <v>16</v>
       </c>
-      <c r="O11" s="56">
+      <c r="O11" s="54">
         <v>0.12570000000000001</v>
       </c>
-      <c r="P11" s="57">
+      <c r="P11" s="55">
         <f t="shared" si="1"/>
         <v>106.845</v>
       </c>
-      <c r="Q11" s="60"/>
-      <c r="R11" s="5"/>
+      <c r="Q11" s="58"/>
+      <c r="R11" s="173"/>
       <c r="S11" s="5"/>
     </row>
-    <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="47">
+    <row r="12" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="45">
         <v>10</v>
       </c>
-      <c r="B12" s="83"/>
+      <c r="B12" s="167"/>
       <c r="C12" s="23" t="s">
         <v>83</v>
       </c>
@@ -2783,10 +2883,10 @@
       <c r="G12" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="H12" s="61" t="s">
+      <c r="H12" s="59" t="s">
         <v>222</v>
       </c>
-      <c r="I12" s="79" t="s">
+      <c r="I12" s="77" t="s">
         <v>216</v>
       </c>
       <c r="J12" s="21" t="s">
@@ -2802,10 +2902,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N12" s="92" t="s">
+      <c r="N12" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O12" s="52">
+      <c r="O12" s="50">
         <v>2.81E-2</v>
       </c>
       <c r="P12" s="9">
@@ -2813,14 +2913,14 @@
         <v>11.802</v>
       </c>
       <c r="Q12" s="10"/>
-      <c r="R12" s="5"/>
+      <c r="R12" s="173"/>
       <c r="S12" s="5"/>
     </row>
-    <row r="13" spans="1:19" s="176" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="47">
+    <row r="13" spans="1:34" s="164" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="45">
         <v>11</v>
       </c>
-      <c r="B13" s="83"/>
+      <c r="B13" s="167"/>
       <c r="C13" s="20" t="s">
         <v>277</v>
       </c>
@@ -2836,10 +2936,10 @@
       <c r="G13" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="H13" s="61" t="s">
+      <c r="H13" s="59" t="s">
         <v>225</v>
       </c>
-      <c r="I13" s="79" t="s">
+      <c r="I13" s="77" t="s">
         <v>216</v>
       </c>
       <c r="J13" s="21" t="s">
@@ -2848,70 +2948,70 @@
       <c r="K13" s="19">
         <v>420</v>
       </c>
-      <c r="L13" s="170">
+      <c r="L13" s="158">
         <v>1</v>
       </c>
       <c r="M13" s="19">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N13" s="171" t="s">
+      <c r="N13" s="159" t="s">
         <v>16</v>
       </c>
-      <c r="O13" s="172">
+      <c r="O13" s="160">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="P13" s="173">
+      <c r="P13" s="161">
         <f t="shared" si="1"/>
         <v>28.14</v>
       </c>
-      <c r="Q13" s="174"/>
-      <c r="R13" s="175"/>
-      <c r="S13" s="175"/>
-    </row>
-    <row r="14" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="47">
+      <c r="Q13" s="162"/>
+      <c r="R13" s="174"/>
+      <c r="S13" s="163"/>
+    </row>
+    <row r="14" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="45">
         <v>12</v>
       </c>
-      <c r="B14" s="87"/>
-      <c r="C14" s="106" t="s">
+      <c r="B14" s="166"/>
+      <c r="C14" s="99" t="s">
         <v>89</v>
       </c>
-      <c r="D14" s="107" t="s">
+      <c r="D14" s="100" t="s">
         <v>90</v>
       </c>
-      <c r="E14" s="107" t="s">
+      <c r="E14" s="100" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="107" t="s">
+      <c r="F14" s="100" t="s">
         <v>91</v>
       </c>
-      <c r="G14" s="108" t="s">
+      <c r="G14" s="101" t="s">
         <v>58</v>
       </c>
-      <c r="H14" s="109" t="s">
+      <c r="H14" s="102" t="s">
         <v>226</v>
       </c>
-      <c r="I14" s="110" t="s">
+      <c r="I14" s="103" t="s">
         <v>216</v>
       </c>
-      <c r="J14" s="111" t="s">
+      <c r="J14" s="104" t="s">
         <v>199</v>
       </c>
-      <c r="K14" s="112">
+      <c r="K14" s="105">
         <v>450</v>
       </c>
       <c r="L14" s="15">
         <v>1</v>
       </c>
-      <c r="M14" s="113">
+      <c r="M14" s="106">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N14" s="80" t="s">
+      <c r="N14" s="78" t="s">
         <v>16</v>
       </c>
-      <c r="O14" s="55">
+      <c r="O14" s="53">
         <v>1.5299999999999999E-2</v>
       </c>
       <c r="P14" s="16">
@@ -2919,41 +3019,41 @@
         <v>6.8849999999999998</v>
       </c>
       <c r="Q14" s="17"/>
-      <c r="R14" s="5"/>
+      <c r="R14" s="173"/>
       <c r="S14" s="5"/>
     </row>
-    <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="47">
+    <row r="15" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="45">
         <v>13</v>
       </c>
-      <c r="B15" s="86" t="s">
+      <c r="B15" s="165" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="102" t="s">
+      <c r="C15" s="95" t="s">
         <v>92</v>
       </c>
-      <c r="D15" s="103" t="s">
+      <c r="D15" s="96" t="s">
         <v>93</v>
       </c>
-      <c r="E15" s="103" t="s">
+      <c r="E15" s="96" t="s">
         <v>94</v>
       </c>
-      <c r="F15" s="103" t="s">
+      <c r="F15" s="96" t="s">
         <v>95</v>
       </c>
-      <c r="G15" s="104" t="s">
+      <c r="G15" s="97" t="s">
         <v>227</v>
       </c>
-      <c r="H15" s="68" t="s">
+      <c r="H15" s="66" t="s">
         <v>228</v>
       </c>
-      <c r="I15" s="75" t="s">
+      <c r="I15" s="73" t="s">
         <v>216</v>
       </c>
-      <c r="J15" s="104" t="s">
+      <c r="J15" s="97" t="s">
         <v>200</v>
       </c>
-      <c r="K15" s="105">
+      <c r="K15" s="98">
         <v>420</v>
       </c>
       <c r="L15" s="1">
@@ -2963,10 +3063,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N15" s="114" t="s">
+      <c r="N15" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="O15" s="51">
+      <c r="O15" s="49">
         <v>2.3599999999999999E-2</v>
       </c>
       <c r="P15" s="3">
@@ -2974,14 +3074,14 @@
         <v>9.911999999999999</v>
       </c>
       <c r="Q15" s="4"/>
-      <c r="R15" s="5"/>
+      <c r="R15" s="173"/>
       <c r="S15" s="5"/>
     </row>
-    <row r="16" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="47">
+    <row r="16" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="45">
         <v>14</v>
       </c>
-      <c r="B16" s="83"/>
+      <c r="B16" s="167"/>
       <c r="C16" s="20" t="s">
         <v>96</v>
       </c>
@@ -2997,10 +3097,10 @@
       <c r="G16" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="H16" s="71" t="s">
+      <c r="H16" s="69" t="s">
         <v>229</v>
       </c>
-      <c r="I16" s="79" t="s">
+      <c r="I16" s="77" t="s">
         <v>216</v>
       </c>
       <c r="J16" s="6" t="s">
@@ -3016,215 +3116,217 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N16" s="92" t="s">
+      <c r="N16" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O16" s="52">
+      <c r="O16" s="50">
         <v>0.1888</v>
       </c>
       <c r="P16" s="9">
         <f t="shared" si="1"/>
         <v>79.295999999999992</v>
       </c>
-      <c r="Q16" s="115"/>
-      <c r="R16" s="5"/>
+      <c r="Q16" s="108"/>
+      <c r="R16" s="173"/>
       <c r="S16" s="5"/>
     </row>
     <row r="17" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="47">
+      <c r="A17" s="45">
         <v>15</v>
       </c>
-      <c r="B17" s="87"/>
-      <c r="C17" s="116" t="s">
+      <c r="B17" s="166"/>
+      <c r="C17" s="109" t="s">
         <v>101</v>
       </c>
-      <c r="D17" s="111" t="s">
+      <c r="D17" s="104" t="s">
         <v>102</v>
       </c>
-      <c r="E17" s="111" t="s">
+      <c r="E17" s="104" t="s">
         <v>276</v>
       </c>
-      <c r="F17" s="111" t="s">
+      <c r="F17" s="104" t="s">
         <v>103</v>
       </c>
-      <c r="G17" s="111" t="s">
+      <c r="G17" s="104" t="s">
         <v>230</v>
       </c>
       <c r="H17" s="14" t="s">
         <v>231</v>
       </c>
-      <c r="I17" s="110" t="s">
+      <c r="I17" s="103" t="s">
         <v>216</v>
       </c>
-      <c r="J17" s="108" t="s">
+      <c r="J17" s="101" t="s">
         <v>200</v>
       </c>
-      <c r="K17" s="112">
+      <c r="K17" s="105">
         <v>420</v>
       </c>
-      <c r="L17" s="44">
+      <c r="L17" s="42">
         <v>1</v>
       </c>
-      <c r="M17" s="113">
+      <c r="M17" s="106">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N17" s="80" t="s">
+      <c r="N17" s="78" t="s">
         <v>16</v>
       </c>
-      <c r="O17" s="65">
+      <c r="O17" s="63">
         <v>2.0299999999999999E-2</v>
       </c>
-      <c r="P17" s="66">
+      <c r="P17" s="64">
         <f t="shared" si="1"/>
         <v>8.5259999999999998</v>
       </c>
-      <c r="Q17" s="67"/>
-      <c r="R17" s="5"/>
+      <c r="Q17" s="65"/>
+      <c r="R17" s="173"/>
       <c r="S17" s="5"/>
     </row>
     <row r="18" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="47">
+      <c r="A18" s="45">
         <v>16</v>
       </c>
-      <c r="B18" s="128" t="s">
+      <c r="B18" s="121" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="140" t="s">
+      <c r="C18" s="133" t="s">
         <v>104</v>
       </c>
-      <c r="D18" s="141" t="s">
+      <c r="D18" s="134" t="s">
         <v>105</v>
       </c>
-      <c r="E18" s="141" t="s">
+      <c r="E18" s="134" t="s">
         <v>106</v>
       </c>
-      <c r="F18" s="141" t="s">
+      <c r="F18" s="134" t="s">
         <v>107</v>
       </c>
-      <c r="G18" s="142" t="s">
+      <c r="G18" s="135" t="s">
         <v>108</v>
       </c>
-      <c r="H18" s="143" t="s">
+      <c r="H18" s="136" t="s">
         <v>216</v>
       </c>
-      <c r="I18" s="144" t="s">
+      <c r="I18" s="137" t="s">
         <v>216</v>
       </c>
-      <c r="J18" s="142" t="s">
+      <c r="J18" s="135" t="s">
         <v>200</v>
       </c>
-      <c r="K18" s="142">
+      <c r="K18" s="135">
         <v>420</v>
       </c>
-      <c r="L18" s="134">
+      <c r="L18" s="127">
         <v>1</v>
       </c>
-      <c r="M18" s="135">
+      <c r="M18" s="128">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N18" s="136" t="s">
+      <c r="N18" s="129" t="s">
         <v>232</v>
       </c>
-      <c r="O18" s="137">
+      <c r="O18" s="130">
         <v>8.158E-2</v>
       </c>
-      <c r="P18" s="138">
+      <c r="P18" s="131">
         <f t="shared" si="1"/>
         <v>34.263599999999997</v>
       </c>
-      <c r="Q18" s="145"/>
-      <c r="R18" s="5"/>
+      <c r="Q18" s="138"/>
+      <c r="R18" s="179">
+        <v>0.189</v>
+      </c>
       <c r="S18" s="5"/>
     </row>
     <row r="19" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="47">
+      <c r="A19" s="45">
         <v>17</v>
       </c>
-      <c r="B19" s="128" t="s">
+      <c r="B19" s="121" t="s">
         <v>210</v>
       </c>
-      <c r="C19" s="129" t="s">
+      <c r="C19" s="122" t="s">
         <v>109</v>
       </c>
-      <c r="D19" s="130" t="s">
+      <c r="D19" s="123" t="s">
         <v>110</v>
       </c>
-      <c r="E19" s="130" t="s">
+      <c r="E19" s="123" t="s">
         <v>25</v>
       </c>
-      <c r="F19" s="130" t="s">
+      <c r="F19" s="123" t="s">
         <v>111</v>
       </c>
-      <c r="G19" s="131" t="s">
+      <c r="G19" s="124" t="s">
         <v>236</v>
       </c>
-      <c r="H19" s="132" t="s">
+      <c r="H19" s="125" t="s">
         <v>233</v>
       </c>
-      <c r="I19" s="133" t="s">
+      <c r="I19" s="126" t="s">
         <v>216</v>
       </c>
-      <c r="J19" s="131" t="s">
+      <c r="J19" s="124" t="s">
         <v>200</v>
       </c>
-      <c r="K19" s="131">
+      <c r="K19" s="124">
         <v>850</v>
       </c>
-      <c r="L19" s="134">
+      <c r="L19" s="127">
         <v>2</v>
       </c>
-      <c r="M19" s="135">
+      <c r="M19" s="128">
         <f t="shared" si="0"/>
         <v>800</v>
       </c>
-      <c r="N19" s="136" t="s">
+      <c r="N19" s="129" t="s">
         <v>16</v>
       </c>
-      <c r="O19" s="137">
+      <c r="O19" s="130">
         <v>4.8399999999999999E-2</v>
       </c>
-      <c r="P19" s="138">
+      <c r="P19" s="131">
         <f t="shared" si="1"/>
         <v>41.14</v>
       </c>
-      <c r="Q19" s="139"/>
-      <c r="R19" s="5"/>
+      <c r="Q19" s="132"/>
+      <c r="R19" s="173"/>
       <c r="S19" s="5"/>
     </row>
     <row r="20" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="47">
+      <c r="A20" s="45">
         <v>18</v>
       </c>
-      <c r="B20" s="86" t="s">
+      <c r="B20" s="165" t="s">
         <v>211</v>
       </c>
-      <c r="C20" s="102" t="s">
+      <c r="C20" s="95" t="s">
         <v>112</v>
       </c>
-      <c r="D20" s="103" t="s">
+      <c r="D20" s="96" t="s">
         <v>113</v>
       </c>
-      <c r="E20" s="103" t="s">
+      <c r="E20" s="96" t="s">
         <v>114</v>
       </c>
-      <c r="F20" s="103" t="s">
+      <c r="F20" s="96" t="s">
         <v>115</v>
       </c>
-      <c r="G20" s="104" t="s">
+      <c r="G20" s="97" t="s">
         <v>234</v>
       </c>
-      <c r="H20" s="70" t="s">
+      <c r="H20" s="68" t="s">
         <v>235</v>
       </c>
-      <c r="I20" s="117" t="s">
+      <c r="I20" s="110" t="s">
         <v>216</v>
       </c>
-      <c r="J20" s="104" t="s">
+      <c r="J20" s="97" t="s">
         <v>200</v>
       </c>
-      <c r="K20" s="104">
+      <c r="K20" s="97">
         <v>2100</v>
       </c>
       <c r="L20" s="1">
@@ -3234,10 +3336,10 @@
         <f t="shared" si="0"/>
         <v>2000</v>
       </c>
-      <c r="N20" s="74" t="s">
+      <c r="N20" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="O20" s="51">
+      <c r="O20" s="49">
         <v>5.1999999999999998E-3</v>
       </c>
       <c r="P20" s="3">
@@ -3245,14 +3347,14 @@
         <v>10.92</v>
       </c>
       <c r="Q20" s="4"/>
-      <c r="R20" s="5"/>
+      <c r="R20" s="173"/>
       <c r="S20" s="5"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="47">
+      <c r="A21" s="45">
         <v>19</v>
       </c>
-      <c r="B21" s="83"/>
+      <c r="B21" s="167"/>
       <c r="C21" s="23" t="s">
         <v>116</v>
       </c>
@@ -3268,10 +3370,10 @@
       <c r="G21" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="H21" s="61" t="s">
+      <c r="H21" s="59" t="s">
         <v>238</v>
       </c>
-      <c r="I21" s="62" t="s">
+      <c r="I21" s="60" t="s">
         <v>216</v>
       </c>
       <c r="J21" s="6" t="s">
@@ -3287,10 +3389,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N21" s="76" t="s">
+      <c r="N21" s="74" t="s">
         <v>16</v>
       </c>
-      <c r="O21" s="52">
+      <c r="O21" s="50">
         <v>3.7900000000000003E-2</v>
       </c>
       <c r="P21" s="9">
@@ -3298,97 +3400,99 @@
         <v>15.918000000000001</v>
       </c>
       <c r="Q21" s="10"/>
-      <c r="R21" s="5"/>
+      <c r="R21" s="173"/>
       <c r="S21" s="5"/>
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="47">
+      <c r="A22" s="45">
         <v>20</v>
       </c>
-      <c r="B22" s="87"/>
-      <c r="C22" s="120" t="s">
+      <c r="B22" s="166"/>
+      <c r="C22" s="113" t="s">
         <v>120</v>
       </c>
-      <c r="D22" s="121" t="s">
+      <c r="D22" s="114" t="s">
         <v>121</v>
       </c>
-      <c r="E22" s="121" t="s">
+      <c r="E22" s="114" t="s">
         <v>23</v>
       </c>
-      <c r="F22" s="121" t="s">
+      <c r="F22" s="114" t="s">
         <v>122</v>
       </c>
-      <c r="G22" s="122" t="s">
+      <c r="G22" s="115" t="s">
         <v>123</v>
       </c>
-      <c r="H22" s="123"/>
-      <c r="I22" s="124"/>
-      <c r="J22" s="122" t="s">
+      <c r="H22" s="116"/>
+      <c r="I22" s="117"/>
+      <c r="J22" s="115" t="s">
         <v>200</v>
       </c>
-      <c r="K22" s="122"/>
-      <c r="L22" s="123">
+      <c r="K22" s="115"/>
+      <c r="L22" s="116">
         <v>1</v>
       </c>
-      <c r="M22" s="125">
+      <c r="M22" s="118">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N22" s="126"/>
-      <c r="O22" s="65"/>
-      <c r="P22" s="66">
+      <c r="N22" s="119"/>
+      <c r="O22" s="63"/>
+      <c r="P22" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q22" s="127"/>
-      <c r="R22" s="5"/>
+      <c r="Q22" s="120"/>
+      <c r="R22" s="179">
+        <v>0.97699999999999998</v>
+      </c>
       <c r="S22" s="5"/>
     </row>
     <row r="23" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="47">
+      <c r="A23" s="45">
         <v>21</v>
       </c>
-      <c r="B23" s="86" t="s">
+      <c r="B23" s="165" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="102" t="s">
+      <c r="C23" s="95" t="s">
         <v>124</v>
       </c>
-      <c r="D23" s="103" t="s">
+      <c r="D23" s="96" t="s">
         <v>125</v>
       </c>
-      <c r="E23" s="103" t="s">
+      <c r="E23" s="96" t="s">
         <v>29</v>
       </c>
-      <c r="F23" s="103" t="s">
+      <c r="F23" s="96" t="s">
         <v>126</v>
       </c>
-      <c r="G23" s="104" t="s">
+      <c r="G23" s="97" t="s">
         <v>58</v>
       </c>
-      <c r="H23" s="70" t="s">
+      <c r="H23" s="68" t="s">
         <v>239</v>
       </c>
-      <c r="I23" s="117" t="s">
+      <c r="I23" s="110" t="s">
         <v>216</v>
       </c>
-      <c r="J23" s="103" t="s">
+      <c r="J23" s="96" t="s">
         <v>28</v>
       </c>
-      <c r="K23" s="105">
+      <c r="K23" s="98">
         <v>6100</v>
       </c>
-      <c r="L23" s="105">
+      <c r="L23" s="98">
         <v>15</v>
       </c>
       <c r="M23" s="2">
         <f t="shared" si="0"/>
         <v>6000</v>
       </c>
-      <c r="N23" s="114" t="s">
+      <c r="N23" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="O23" s="51">
+      <c r="O23" s="49">
         <v>1.4E-3</v>
       </c>
       <c r="P23" s="3">
@@ -3396,14 +3500,14 @@
         <v>8.5399999999999991</v>
       </c>
       <c r="Q23" s="4"/>
-      <c r="R23" s="5"/>
+      <c r="R23" s="173"/>
       <c r="S23" s="5"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="47">
+      <c r="A24" s="45">
         <v>22</v>
       </c>
-      <c r="B24" s="83"/>
+      <c r="B24" s="167"/>
       <c r="C24" s="23" t="s">
         <v>127</v>
       </c>
@@ -3419,10 +3523,10 @@
       <c r="G24" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="H24" s="61" t="s">
+      <c r="H24" s="59" t="s">
         <v>240</v>
       </c>
-      <c r="I24" s="62" t="s">
+      <c r="I24" s="60" t="s">
         <v>216</v>
       </c>
       <c r="J24" s="21" t="s">
@@ -3438,10 +3542,10 @@
         <f t="shared" si="0"/>
         <v>1200</v>
       </c>
-      <c r="N24" s="92" t="s">
+      <c r="N24" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O24" s="52">
+      <c r="O24" s="50">
         <v>1.1000000000000001E-3</v>
       </c>
       <c r="P24" s="9">
@@ -3449,14 +3553,14 @@
         <v>1.4300000000000002</v>
       </c>
       <c r="Q24" s="10"/>
-      <c r="R24" s="5"/>
+      <c r="R24" s="173"/>
       <c r="S24" s="5"/>
     </row>
     <row r="25" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="47">
+      <c r="A25" s="45">
         <v>23</v>
       </c>
-      <c r="B25" s="83"/>
+      <c r="B25" s="167"/>
       <c r="C25" s="23" t="s">
         <v>130</v>
       </c>
@@ -3472,10 +3576,10 @@
       <c r="G25" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="H25" s="61" t="s">
+      <c r="H25" s="59" t="s">
         <v>241</v>
       </c>
-      <c r="I25" s="62" t="s">
+      <c r="I25" s="60" t="s">
         <v>216</v>
       </c>
       <c r="J25" s="21" t="s">
@@ -3484,32 +3588,32 @@
       <c r="K25" s="19">
         <v>1300</v>
       </c>
-      <c r="L25" s="59">
+      <c r="L25" s="57">
         <v>3</v>
       </c>
       <c r="M25" s="8">
         <f t="shared" si="0"/>
         <v>1200</v>
       </c>
-      <c r="N25" s="95" t="s">
+      <c r="N25" s="88" t="s">
         <v>16</v>
       </c>
-      <c r="O25" s="63">
+      <c r="O25" s="61">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="P25" s="64">
+      <c r="P25" s="62">
         <f t="shared" si="1"/>
         <v>1.17</v>
       </c>
-      <c r="Q25" s="69"/>
-      <c r="R25" s="5"/>
+      <c r="Q25" s="67"/>
+      <c r="R25" s="173"/>
       <c r="S25" s="5"/>
     </row>
     <row r="26" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="47">
+      <c r="A26" s="45">
         <v>24</v>
       </c>
-      <c r="B26" s="83"/>
+      <c r="B26" s="167"/>
       <c r="C26" s="23" t="s">
         <v>133</v>
       </c>
@@ -3525,10 +3629,10 @@
       <c r="G26" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="H26" s="61" t="s">
+      <c r="H26" s="59" t="s">
         <v>242</v>
       </c>
-      <c r="I26" s="62" t="s">
+      <c r="I26" s="60" t="s">
         <v>216</v>
       </c>
       <c r="J26" s="21" t="s">
@@ -3544,10 +3648,10 @@
         <f t="shared" si="0"/>
         <v>2400</v>
       </c>
-      <c r="N26" s="92" t="s">
+      <c r="N26" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O26" s="52">
+      <c r="O26" s="50">
         <v>1E-3</v>
       </c>
       <c r="P26" s="9">
@@ -3555,14 +3659,14 @@
         <v>2.5</v>
       </c>
       <c r="Q26" s="10"/>
-      <c r="R26" s="5"/>
+      <c r="R26" s="173"/>
       <c r="S26" s="5"/>
     </row>
     <row r="27" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="47">
+      <c r="A27" s="45">
         <v>25</v>
       </c>
-      <c r="B27" s="83"/>
+      <c r="B27" s="167"/>
       <c r="C27" s="23" t="s">
         <v>136</v>
       </c>
@@ -3578,10 +3682,10 @@
       <c r="G27" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="H27" s="61" t="s">
+      <c r="H27" s="59" t="s">
         <v>243</v>
       </c>
-      <c r="I27" s="62" t="s">
+      <c r="I27" s="60" t="s">
         <v>216</v>
       </c>
       <c r="J27" s="21" t="s">
@@ -3597,10 +3701,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N27" s="92" t="s">
+      <c r="N27" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O27" s="52">
+      <c r="O27" s="50">
         <v>1.38E-2</v>
       </c>
       <c r="P27" s="9">
@@ -3608,14 +3712,14 @@
         <v>5.7960000000000003</v>
       </c>
       <c r="Q27" s="10"/>
-      <c r="R27" s="5"/>
+      <c r="R27" s="173"/>
       <c r="S27" s="5"/>
     </row>
     <row r="28" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="47">
+      <c r="A28" s="45">
         <v>26</v>
       </c>
-      <c r="B28" s="83"/>
+      <c r="B28" s="167"/>
       <c r="C28" s="23" t="s">
         <v>140</v>
       </c>
@@ -3631,10 +3735,10 @@
       <c r="G28" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="H28" s="61" t="s">
+      <c r="H28" s="59" t="s">
         <v>245</v>
       </c>
-      <c r="I28" s="62" t="s">
+      <c r="I28" s="60" t="s">
         <v>216</v>
       </c>
       <c r="J28" s="21" t="s">
@@ -3650,10 +3754,10 @@
         <f t="shared" si="0"/>
         <v>800</v>
       </c>
-      <c r="N28" s="92" t="s">
+      <c r="N28" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O28" s="52">
+      <c r="O28" s="50">
         <v>3.0700000000000002E-2</v>
       </c>
       <c r="P28" s="9">
@@ -3661,14 +3765,14 @@
         <v>26.095000000000002</v>
       </c>
       <c r="Q28" s="10"/>
-      <c r="R28" s="5"/>
+      <c r="R28" s="173"/>
       <c r="S28" s="5"/>
     </row>
     <row r="29" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="47">
+      <c r="A29" s="45">
         <v>27</v>
       </c>
-      <c r="B29" s="83"/>
+      <c r="B29" s="167"/>
       <c r="C29" s="23" t="s">
         <v>144</v>
       </c>
@@ -3684,7 +3788,7 @@
       <c r="G29" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="H29" s="61" t="s">
+      <c r="H29" s="59" t="s">
         <v>270</v>
       </c>
       <c r="I29" s="11" t="s">
@@ -3703,10 +3807,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N29" s="92" t="s">
+      <c r="N29" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O29" s="52">
+      <c r="O29" s="50">
         <v>8.2400000000000001E-2</v>
       </c>
       <c r="P29" s="9">
@@ -3714,14 +3818,14 @@
         <v>34.607999999999997</v>
       </c>
       <c r="Q29" s="10"/>
-      <c r="R29" s="5"/>
+      <c r="R29" s="173"/>
       <c r="S29" s="5"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="47">
+      <c r="A30" s="45">
         <v>28</v>
       </c>
-      <c r="B30" s="83"/>
+      <c r="B30" s="167"/>
       <c r="C30" s="23" t="s">
         <v>147</v>
       </c>
@@ -3737,10 +3841,10 @@
       <c r="G30" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="H30" s="61" t="s">
+      <c r="H30" s="59" t="s">
         <v>246</v>
       </c>
-      <c r="I30" s="62" t="s">
+      <c r="I30" s="60" t="s">
         <v>216</v>
       </c>
       <c r="J30" s="21" t="s">
@@ -3756,10 +3860,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N30" s="92" t="s">
+      <c r="N30" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O30" s="52">
+      <c r="O30" s="50">
         <v>2.8E-3</v>
       </c>
       <c r="P30" s="9">
@@ -3767,159 +3871,167 @@
         <v>1.4</v>
       </c>
       <c r="Q30" s="10"/>
-      <c r="R30" s="5"/>
+      <c r="R30" s="173"/>
       <c r="S30" s="5"/>
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="47">
+      <c r="A31" s="45">
         <v>29</v>
       </c>
-      <c r="B31" s="87"/>
-      <c r="C31" s="106" t="s">
+      <c r="B31" s="166"/>
+      <c r="C31" s="99" t="s">
         <v>273</v>
       </c>
-      <c r="D31" s="111" t="s">
+      <c r="D31" s="104" t="s">
         <v>150</v>
       </c>
-      <c r="E31" s="111" t="s">
+      <c r="E31" s="104" t="s">
         <v>29</v>
       </c>
-      <c r="F31" s="111" t="s">
+      <c r="F31" s="104" t="s">
         <v>151</v>
       </c>
-      <c r="G31" s="108" t="s">
+      <c r="G31" s="101" t="s">
         <v>58</v>
       </c>
-      <c r="H31" s="109" t="s">
+      <c r="H31" s="102" t="s">
         <v>248</v>
       </c>
-      <c r="I31" s="118" t="s">
+      <c r="I31" s="111" t="s">
         <v>216</v>
       </c>
-      <c r="J31" s="111" t="s">
+      <c r="J31" s="104" t="s">
         <v>208</v>
       </c>
-      <c r="K31" s="112">
+      <c r="K31" s="105">
         <v>3300</v>
       </c>
       <c r="L31" s="15">
         <v>8</v>
       </c>
-      <c r="M31" s="113">
+      <c r="M31" s="106">
         <f t="shared" si="0"/>
         <v>3200</v>
       </c>
-      <c r="N31" s="119" t="s">
+      <c r="N31" s="112" t="s">
         <v>16</v>
       </c>
-      <c r="O31" s="55">
+      <c r="O31" s="53">
         <v>1.5E-3</v>
       </c>
       <c r="P31" s="16">
-        <f t="shared" si="1"/>
+        <f>O31*K31</f>
         <v>4.95</v>
       </c>
       <c r="Q31" s="17"/>
-      <c r="R31" s="5"/>
+      <c r="R31" s="173"/>
       <c r="S31" s="5"/>
     </row>
     <row r="32" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="47">
+      <c r="A32" s="45">
         <v>30</v>
       </c>
-      <c r="B32" s="128" t="s">
+      <c r="B32" s="121" t="s">
         <v>212</v>
       </c>
-      <c r="C32" s="140" t="s">
+      <c r="C32" s="133" t="s">
         <v>152</v>
       </c>
-      <c r="D32" s="141" t="s">
+      <c r="D32" s="134" t="s">
         <v>153</v>
       </c>
-      <c r="E32" s="141" t="s">
+      <c r="E32" s="134" t="s">
         <v>23</v>
       </c>
-      <c r="F32" s="141" t="s">
+      <c r="F32" s="134" t="s">
         <v>154</v>
       </c>
-      <c r="G32" s="142" t="s">
+      <c r="G32" s="135" t="s">
         <v>249</v>
       </c>
-      <c r="H32" s="143" t="s">
+      <c r="H32" s="136" t="s">
         <v>216</v>
       </c>
-      <c r="I32" s="144" t="s">
+      <c r="I32" s="137" t="s">
         <v>216</v>
       </c>
-      <c r="J32" s="142"/>
-      <c r="K32" s="142">
+      <c r="J32" s="135"/>
+      <c r="K32" s="135">
         <v>420</v>
       </c>
-      <c r="L32" s="134">
+      <c r="L32" s="127">
         <v>1</v>
       </c>
-      <c r="M32" s="135">
+      <c r="M32" s="128">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N32" s="157" t="s">
+      <c r="N32" s="149" t="s">
         <v>232</v>
       </c>
-      <c r="O32" s="137">
+      <c r="O32" s="130">
         <v>0.49325000000000002</v>
       </c>
-      <c r="P32" s="138">
+      <c r="P32" s="131">
         <f t="shared" si="1"/>
         <v>207.16500000000002</v>
       </c>
-      <c r="Q32" s="139"/>
-      <c r="R32" s="5"/>
+      <c r="Q32" s="132"/>
+      <c r="R32" s="179">
+        <v>0.441</v>
+      </c>
       <c r="S32" s="5"/>
     </row>
-    <row r="33" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="47">
+    <row r="33" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="45">
         <v>31</v>
       </c>
-      <c r="B33" s="86" t="s">
+      <c r="B33" s="165" t="s">
         <v>30</v>
       </c>
-      <c r="C33" s="146" t="s">
+      <c r="C33" s="139" t="s">
         <v>155</v>
       </c>
-      <c r="D33" s="147" t="s">
+      <c r="D33" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="E33" s="147"/>
-      <c r="F33" s="147" t="s">
+      <c r="E33" s="140"/>
+      <c r="F33" s="140" t="s">
         <v>156</v>
       </c>
-      <c r="G33" s="148"/>
-      <c r="H33" s="149"/>
-      <c r="I33" s="150"/>
-      <c r="J33" s="148"/>
-      <c r="K33" s="148"/>
-      <c r="L33" s="149">
+      <c r="G33" s="141"/>
+      <c r="H33" s="142"/>
+      <c r="I33" s="143"/>
+      <c r="J33" s="141"/>
+      <c r="K33" s="141"/>
+      <c r="L33" s="142">
         <v>1</v>
       </c>
-      <c r="M33" s="151">
-        <f t="shared" si="0"/>
-        <v>400</v>
-      </c>
-      <c r="N33" s="152"/>
-      <c r="O33" s="51"/>
+      <c r="M33" s="144">
+        <f>L33*900</f>
+        <v>900</v>
+      </c>
+      <c r="N33" s="178" t="s">
+        <v>281</v>
+      </c>
+      <c r="O33" s="177">
+        <v>21.26</v>
+      </c>
       <c r="P33" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>O33*M33</f>
+        <v>19134</v>
       </c>
       <c r="Q33" s="4"/>
-      <c r="R33" s="5"/>
+      <c r="R33" s="179">
+        <v>21.26</v>
+      </c>
       <c r="S33" s="5"/>
     </row>
     <row r="34" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="47">
+      <c r="A34" s="45">
         <v>32</v>
       </c>
-      <c r="B34" s="83"/>
+      <c r="B34" s="167"/>
       <c r="C34" s="23" t="s">
         <v>157</v>
       </c>
@@ -3935,10 +4047,10 @@
       <c r="G34" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H34" s="61" t="s">
+      <c r="H34" s="59" t="s">
         <v>250</v>
       </c>
-      <c r="I34" s="62" t="s">
+      <c r="I34" s="60" t="s">
         <v>216</v>
       </c>
       <c r="J34" s="6" t="s">
@@ -3954,10 +4066,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N34" s="76" t="s">
+      <c r="N34" s="74" t="s">
         <v>16</v>
       </c>
-      <c r="O34" s="52">
+      <c r="O34" s="50">
         <v>0.2868</v>
       </c>
       <c r="P34" s="9">
@@ -3965,39 +4077,39 @@
         <v>120.456</v>
       </c>
       <c r="Q34" s="10"/>
-      <c r="R34" s="5"/>
+      <c r="R34" s="173"/>
       <c r="S34" s="5"/>
     </row>
     <row r="35" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="47">
+      <c r="A35" s="45">
         <v>33</v>
       </c>
-      <c r="B35" s="83"/>
-      <c r="C35" s="101" t="s">
+      <c r="B35" s="167"/>
+      <c r="C35" s="94" t="s">
         <v>271</v>
       </c>
-      <c r="D35" s="97" t="s">
+      <c r="D35" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="E35" s="97" t="s">
+      <c r="E35" s="90" t="s">
         <v>161</v>
       </c>
-      <c r="F35" s="97" t="s">
+      <c r="F35" s="90" t="s">
         <v>162</v>
       </c>
-      <c r="G35" s="98" t="s">
+      <c r="G35" s="91" t="s">
         <v>163</v>
       </c>
-      <c r="H35" s="99" t="s">
+      <c r="H35" s="92" t="s">
         <v>216</v>
       </c>
-      <c r="I35" s="100" t="s">
+      <c r="I35" s="93" t="s">
         <v>216</v>
       </c>
-      <c r="J35" s="98" t="s">
+      <c r="J35" s="91" t="s">
         <v>200</v>
       </c>
-      <c r="K35" s="98">
+      <c r="K35" s="91">
         <v>420</v>
       </c>
       <c r="L35" s="7">
@@ -4007,10 +4119,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N35" s="76" t="s">
+      <c r="N35" s="74" t="s">
         <v>272</v>
       </c>
-      <c r="O35" s="52">
+      <c r="O35" s="50">
         <v>1</v>
       </c>
       <c r="P35" s="9">
@@ -4018,67 +4130,71 @@
         <v>420</v>
       </c>
       <c r="Q35" s="10"/>
-      <c r="R35" s="5"/>
+      <c r="R35" s="179">
+        <v>2.8347000000000002</v>
+      </c>
       <c r="S35" s="5"/>
     </row>
     <row r="36" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="47">
+      <c r="A36" s="45">
         <v>34</v>
       </c>
-      <c r="B36" s="83"/>
-      <c r="C36" s="96" t="s">
+      <c r="B36" s="167"/>
+      <c r="C36" s="89" t="s">
         <v>164</v>
       </c>
-      <c r="D36" s="97" t="s">
+      <c r="D36" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="E36" s="97" t="s">
+      <c r="E36" s="90" t="s">
         <v>158</v>
       </c>
-      <c r="F36" s="97" t="s">
+      <c r="F36" s="90" t="s">
         <v>165</v>
       </c>
-      <c r="G36" s="98" t="s">
+      <c r="G36" s="91" t="s">
         <v>166</v>
       </c>
-      <c r="H36" s="99" t="s">
+      <c r="H36" s="92" t="s">
         <v>216</v>
       </c>
-      <c r="I36" s="100" t="s">
+      <c r="I36" s="93" t="s">
         <v>216</v>
       </c>
-      <c r="J36" s="98" t="s">
+      <c r="J36" s="91" t="s">
         <v>200</v>
       </c>
-      <c r="K36" s="98">
+      <c r="K36" s="91">
         <v>420</v>
       </c>
-      <c r="L36" s="41">
+      <c r="L36" s="40">
         <v>1</v>
       </c>
       <c r="M36" s="8">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N36" s="93" t="s">
+      <c r="N36" s="86" t="s">
         <v>272</v>
       </c>
-      <c r="O36" s="94">
+      <c r="O36" s="87">
         <v>5</v>
       </c>
-      <c r="P36" s="54">
+      <c r="P36" s="52">
         <f t="shared" si="1"/>
         <v>2100</v>
       </c>
       <c r="Q36" s="13"/>
-      <c r="R36" s="5"/>
+      <c r="R36" s="179">
+        <v>2.7559999999999998</v>
+      </c>
       <c r="S36" s="5"/>
     </row>
     <row r="37" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="47">
+      <c r="A37" s="45">
         <v>35</v>
       </c>
-      <c r="B37" s="83"/>
+      <c r="B37" s="167"/>
       <c r="C37" s="23" t="s">
         <v>167</v>
       </c>
@@ -4094,10 +4210,10 @@
       <c r="G37" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="H37" s="61" t="s">
+      <c r="H37" s="59" t="s">
         <v>251</v>
       </c>
-      <c r="I37" s="62" t="s">
+      <c r="I37" s="60" t="s">
         <v>216</v>
       </c>
       <c r="J37" s="6" t="s">
@@ -4113,10 +4229,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N37" s="92" t="s">
+      <c r="N37" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O37" s="52">
+      <c r="O37" s="50">
         <v>0.85660000000000003</v>
       </c>
       <c r="P37" s="9">
@@ -4124,14 +4240,14 @@
         <v>359.77199999999999</v>
       </c>
       <c r="Q37" s="10"/>
-      <c r="R37" s="5"/>
+      <c r="R37" s="173"/>
       <c r="S37" s="5"/>
     </row>
     <row r="38" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="47">
+      <c r="A38" s="45">
         <v>36</v>
       </c>
-      <c r="B38" s="83"/>
+      <c r="B38" s="167"/>
       <c r="C38" s="23" t="s">
         <v>172</v>
       </c>
@@ -4147,10 +4263,10 @@
       <c r="G38" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="H38" s="61" t="s">
+      <c r="H38" s="59" t="s">
         <v>253</v>
       </c>
-      <c r="I38" s="62" t="s">
+      <c r="I38" s="60" t="s">
         <v>216</v>
       </c>
       <c r="J38" s="6" t="s">
@@ -4166,10 +4282,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N38" s="92" t="s">
+      <c r="N38" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O38" s="52">
+      <c r="O38" s="50">
         <v>0.18229999999999999</v>
       </c>
       <c r="P38" s="9">
@@ -4177,84 +4293,84 @@
         <v>76.566000000000003</v>
       </c>
       <c r="Q38" s="10"/>
-      <c r="R38" s="5"/>
+      <c r="R38" s="173"/>
       <c r="S38" s="5"/>
     </row>
     <row r="39" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="47">
+      <c r="A39" s="45">
         <v>37</v>
       </c>
-      <c r="B39" s="87"/>
-      <c r="C39" s="106" t="s">
+      <c r="B39" s="166"/>
+      <c r="C39" s="99" t="s">
         <v>255</v>
       </c>
-      <c r="D39" s="111" t="s">
+      <c r="D39" s="104" t="s">
         <v>35</v>
       </c>
-      <c r="E39" s="107" t="s">
+      <c r="E39" s="100" t="s">
         <v>254</v>
       </c>
-      <c r="F39" s="111" t="s">
+      <c r="F39" s="104" t="s">
         <v>174</v>
       </c>
-      <c r="G39" s="108" t="s">
+      <c r="G39" s="101" t="s">
         <v>256</v>
       </c>
-      <c r="H39" s="109" t="s">
+      <c r="H39" s="102" t="s">
         <v>257</v>
       </c>
-      <c r="I39" s="118" t="s">
+      <c r="I39" s="111" t="s">
         <v>216</v>
       </c>
-      <c r="J39" s="108"/>
-      <c r="K39" s="108">
+      <c r="J39" s="101"/>
+      <c r="K39" s="101">
         <v>420</v>
       </c>
-      <c r="L39" s="44">
+      <c r="L39" s="42">
         <v>1</v>
       </c>
-      <c r="M39" s="113">
+      <c r="M39" s="106">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N39" s="153" t="s">
+      <c r="N39" s="145" t="s">
         <v>16</v>
       </c>
-      <c r="O39" s="154">
+      <c r="O39" s="146">
         <v>0.11550000000000001</v>
       </c>
-      <c r="P39" s="155">
+      <c r="P39" s="147">
         <f t="shared" si="1"/>
         <v>48.510000000000005</v>
       </c>
-      <c r="Q39" s="156"/>
-      <c r="R39" s="5"/>
+      <c r="Q39" s="148"/>
+      <c r="R39" s="173"/>
       <c r="S39" s="5"/>
     </row>
     <row r="40" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="47">
+      <c r="A40" s="45">
         <v>38</v>
       </c>
-      <c r="B40" s="86" t="s">
+      <c r="B40" s="165" t="s">
         <v>213</v>
       </c>
-      <c r="C40" s="160" t="s">
+      <c r="C40" s="152" t="s">
         <v>175</v>
       </c>
-      <c r="D40" s="147" t="s">
+      <c r="D40" s="140" t="s">
         <v>176</v>
       </c>
-      <c r="E40" s="147" t="s">
+      <c r="E40" s="140" t="s">
         <v>23</v>
       </c>
-      <c r="F40" s="147" t="s">
+      <c r="F40" s="140" t="s">
         <v>177</v>
       </c>
-      <c r="G40" s="147"/>
-      <c r="H40" s="149"/>
-      <c r="I40" s="148"/>
-      <c r="J40" s="148"/>
-      <c r="K40" s="148"/>
+      <c r="G40" s="140"/>
+      <c r="H40" s="142"/>
+      <c r="I40" s="141"/>
+      <c r="J40" s="141"/>
+      <c r="K40" s="141"/>
       <c r="L40" s="1">
         <v>1</v>
       </c>
@@ -4262,87 +4378,95 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N40" s="161"/>
-      <c r="O40" s="51"/>
+      <c r="N40" s="153"/>
+      <c r="O40" s="49"/>
       <c r="P40" s="3">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q40" s="162"/>
-      <c r="R40" s="5"/>
+      <c r="Q40" s="154"/>
+      <c r="R40" s="179" t="s">
+        <v>279</v>
+      </c>
       <c r="S40" s="5"/>
     </row>
     <row r="41" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="47">
+      <c r="A41" s="45">
         <v>39</v>
       </c>
-      <c r="B41" s="87"/>
-      <c r="C41" s="163" t="s">
+      <c r="B41" s="166"/>
+      <c r="C41" s="155" t="s">
         <v>178</v>
       </c>
-      <c r="D41" s="121" t="s">
+      <c r="D41" s="114" t="s">
         <v>179</v>
       </c>
-      <c r="E41" s="121" t="s">
+      <c r="E41" s="114" t="s">
         <v>23</v>
       </c>
-      <c r="F41" s="121" t="s">
+      <c r="F41" s="114" t="s">
         <v>180</v>
       </c>
-      <c r="G41" s="121"/>
-      <c r="H41" s="123"/>
-      <c r="I41" s="122"/>
-      <c r="J41" s="122"/>
-      <c r="K41" s="122"/>
+      <c r="G41" s="114"/>
+      <c r="H41" s="116"/>
+      <c r="I41" s="115"/>
+      <c r="J41" s="115"/>
+      <c r="K41" s="115"/>
       <c r="L41" s="15">
         <v>1</v>
       </c>
-      <c r="M41" s="113">
+      <c r="M41" s="106">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N41" s="164"/>
-      <c r="O41" s="55"/>
+      <c r="N41" s="176" t="s">
+        <v>280</v>
+      </c>
+      <c r="O41" s="177">
+        <v>0.86619999999999997</v>
+      </c>
       <c r="P41" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q41" s="165"/>
-      <c r="R41" s="5"/>
+        <f>O41*M41</f>
+        <v>346.47999999999996</v>
+      </c>
+      <c r="Q41" s="156"/>
+      <c r="R41" s="179">
+        <v>0.86619999999999997</v>
+      </c>
       <c r="S41" s="5"/>
     </row>
     <row r="42" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="47">
+      <c r="A42" s="45">
         <v>40</v>
       </c>
-      <c r="B42" s="86" t="s">
+      <c r="B42" s="165" t="s">
         <v>37</v>
       </c>
-      <c r="C42" s="158" t="s">
+      <c r="C42" s="150" t="s">
         <v>181</v>
       </c>
-      <c r="D42" s="103" t="s">
+      <c r="D42" s="96" t="s">
         <v>182</v>
       </c>
-      <c r="E42" s="103" t="s">
+      <c r="E42" s="96" t="s">
         <v>183</v>
       </c>
-      <c r="F42" s="103" t="s">
+      <c r="F42" s="96" t="s">
         <v>184</v>
       </c>
-      <c r="G42" s="104" t="s">
+      <c r="G42" s="97" t="s">
         <v>185</v>
       </c>
       <c r="H42" s="18" t="s">
         <v>274</v>
       </c>
-      <c r="I42" s="104" t="s">
+      <c r="I42" s="97" t="s">
         <v>275</v>
       </c>
-      <c r="J42" s="104" t="s">
+      <c r="J42" s="97" t="s">
         <v>200</v>
       </c>
-      <c r="K42" s="104">
+      <c r="K42" s="97">
         <v>420</v>
       </c>
       <c r="L42" s="1">
@@ -4352,10 +4476,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N42" s="114" t="s">
+      <c r="N42" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="O42" s="51">
+      <c r="O42" s="49">
         <v>0.12889999999999999</v>
       </c>
       <c r="P42" s="3">
@@ -4363,15 +4487,15 @@
         <v>54.137999999999991</v>
       </c>
       <c r="Q42" s="4"/>
-      <c r="R42" s="5"/>
+      <c r="R42" s="173"/>
       <c r="S42" s="5"/>
     </row>
     <row r="43" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="47">
+      <c r="A43" s="45">
         <v>41</v>
       </c>
-      <c r="B43" s="83"/>
-      <c r="C43" s="73" t="s">
+      <c r="B43" s="167"/>
+      <c r="C43" s="71" t="s">
         <v>38</v>
       </c>
       <c r="D43" s="21" t="s">
@@ -4389,7 +4513,7 @@
       <c r="H43" s="22" t="s">
         <v>258</v>
       </c>
-      <c r="I43" s="62" t="s">
+      <c r="I43" s="60" t="s">
         <v>216</v>
       </c>
       <c r="J43" s="6" t="s">
@@ -4405,10 +4529,10 @@
         <f t="shared" si="0"/>
         <v>800</v>
       </c>
-      <c r="N43" s="92" t="s">
+      <c r="N43" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O43" s="52">
+      <c r="O43" s="50">
         <v>7.0599999999999996E-2</v>
       </c>
       <c r="P43" s="9">
@@ -4416,15 +4540,15 @@
         <v>60.01</v>
       </c>
       <c r="Q43" s="10"/>
-      <c r="R43" s="5"/>
+      <c r="R43" s="173"/>
       <c r="S43" s="5"/>
     </row>
     <row r="44" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="47">
+      <c r="A44" s="45">
         <v>42</v>
       </c>
-      <c r="B44" s="83"/>
-      <c r="C44" s="169" t="s">
+      <c r="B44" s="167"/>
+      <c r="C44" s="157" t="s">
         <v>189</v>
       </c>
       <c r="D44" s="12" t="s">
@@ -4442,7 +4566,7 @@
       <c r="H44" s="22" t="s">
         <v>260</v>
       </c>
-      <c r="I44" s="62" t="s">
+      <c r="I44" s="60" t="s">
         <v>216</v>
       </c>
       <c r="J44" s="6" t="s">
@@ -4458,10 +4582,10 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="N44" s="92" t="s">
+      <c r="N44" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="O44" s="52">
+      <c r="O44" s="50">
         <v>1.8800000000000001E-2</v>
       </c>
       <c r="P44" s="9">
@@ -4469,14 +4593,14 @@
         <v>8.2720000000000002</v>
       </c>
       <c r="Q44" s="10"/>
-      <c r="R44" s="5"/>
+      <c r="R44" s="173"/>
       <c r="S44" s="5"/>
     </row>
     <row r="45" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="47">
+      <c r="A45" s="45">
         <v>43</v>
       </c>
-      <c r="B45" s="83"/>
+      <c r="B45" s="167"/>
       <c r="C45" s="25" t="s">
         <v>43</v>
       </c>
@@ -4510,24 +4634,24 @@
       <c r="Q45" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="R45" s="5"/>
+      <c r="R45" s="173"/>
       <c r="S45" s="5"/>
     </row>
     <row r="46" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="47">
+      <c r="A46" s="45">
         <v>44</v>
       </c>
-      <c r="B46" s="87"/>
+      <c r="B46" s="166"/>
       <c r="C46" s="32" t="s">
         <v>40</v>
       </c>
       <c r="D46" s="33" t="s">
         <v>194</v>
       </c>
-      <c r="E46" s="88" t="s">
+      <c r="E46" s="81" t="s">
         <v>41</v>
       </c>
-      <c r="F46" s="89" t="s">
+      <c r="F46" s="82" t="s">
         <v>41</v>
       </c>
       <c r="G46" s="34"/>
@@ -4538,46 +4662,49 @@
       <c r="L46" s="35">
         <v>6</v>
       </c>
-      <c r="M46" s="159">
+      <c r="M46" s="151">
         <f t="shared" si="0"/>
         <v>2400</v>
       </c>
-      <c r="N46" s="45"/>
-      <c r="O46" s="90"/>
-      <c r="P46" s="90">
+      <c r="N46" s="43"/>
+      <c r="O46" s="83"/>
+      <c r="P46" s="83">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q46" s="36" t="s">
         <v>42</v>
       </c>
-      <c r="R46" s="5"/>
+      <c r="R46" s="175"/>
       <c r="S46" s="5"/>
     </row>
     <row r="47" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47"/>
-      <c r="L47" s="84" t="s">
+      <c r="L47" s="180" t="s">
         <v>45</v>
       </c>
-      <c r="M47" s="84"/>
-      <c r="N47" s="84"/>
-      <c r="O47" s="84"/>
-      <c r="P47" s="43">
+      <c r="M47" s="181"/>
+      <c r="N47" s="181"/>
+      <c r="O47" s="181"/>
+      <c r="P47" s="182">
         <f>SUM(P3:P46)</f>
-        <v>4217.1196</v>
+        <v>23697.599599999994</v>
       </c>
       <c r="R47" s="5"/>
       <c r="S47" s="5"/>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48"/>
-      <c r="L48" s="85" t="s">
+      <c r="L48" s="183" t="s">
         <v>46</v>
       </c>
-      <c r="M48" s="85"/>
-      <c r="N48" s="85"/>
-      <c r="O48" s="85"/>
-      <c r="P48" s="38"/>
+      <c r="M48" s="184"/>
+      <c r="N48" s="184"/>
+      <c r="O48" s="184"/>
+      <c r="P48" s="185">
+        <f>P47/400</f>
+        <v>59.243998999999988</v>
+      </c>
       <c r="R48" s="5"/>
       <c r="S48" s="5"/>
     </row>
@@ -4647,15 +4774,16 @@
       <c r="S61" s="5"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="H62" s="82"/>
-      <c r="Q62" s="42"/>
+      <c r="H62" s="80"/>
+      <c r="Q62" s="41"/>
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="H63" s="82"/>
-      <c r="Q63" s="42"/>
+      <c r="H63" s="80"/>
+      <c r="Q63" s="41"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
+    <mergeCell ref="R1:AH1"/>
     <mergeCell ref="B40:B41"/>
     <mergeCell ref="B42:B46"/>
     <mergeCell ref="L47:O47"/>
@@ -4880,44 +5008,44 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="N3" r:id="rId1"/>
-    <hyperlink ref="N4" r:id="rId2"/>
-    <hyperlink ref="N5" r:id="rId3"/>
-    <hyperlink ref="N10" r:id="rId4"/>
-    <hyperlink ref="N11" r:id="rId5"/>
-    <hyperlink ref="N12" r:id="rId6"/>
-    <hyperlink ref="N13" r:id="rId7"/>
-    <hyperlink ref="N14" r:id="rId8"/>
-    <hyperlink ref="N15" r:id="rId9"/>
-    <hyperlink ref="N16" r:id="rId10"/>
-    <hyperlink ref="N17" r:id="rId11"/>
-    <hyperlink ref="N18" r:id="rId12"/>
-    <hyperlink ref="N19" r:id="rId13"/>
-    <hyperlink ref="N20" r:id="rId14"/>
-    <hyperlink ref="N21" r:id="rId15"/>
-    <hyperlink ref="N23" r:id="rId16"/>
-    <hyperlink ref="N25" r:id="rId17"/>
-    <hyperlink ref="N24" r:id="rId18"/>
-    <hyperlink ref="N26" r:id="rId19"/>
-    <hyperlink ref="N27" r:id="rId20"/>
-    <hyperlink ref="N28" r:id="rId21"/>
-    <hyperlink ref="N30" r:id="rId22"/>
-    <hyperlink ref="N31" r:id="rId23"/>
-    <hyperlink ref="N32" r:id="rId24"/>
-    <hyperlink ref="N34" r:id="rId25"/>
-    <hyperlink ref="N37" r:id="rId26"/>
-    <hyperlink ref="N38" r:id="rId27"/>
-    <hyperlink ref="N39" r:id="rId28"/>
-    <hyperlink ref="N43" r:id="rId29"/>
-    <hyperlink ref="N44" r:id="rId30"/>
-    <hyperlink ref="N6" r:id="rId31"/>
-    <hyperlink ref="N7" r:id="rId32"/>
-    <hyperlink ref="N8" r:id="rId33"/>
-    <hyperlink ref="N9" r:id="rId34"/>
-    <hyperlink ref="N29" r:id="rId35"/>
-    <hyperlink ref="N35" r:id="rId36"/>
-    <hyperlink ref="N36" r:id="rId37"/>
-    <hyperlink ref="N42" r:id="rId38"/>
+    <hyperlink ref="N3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="N4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="N5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="N10" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="N11" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="N12" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="N13" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="N14" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="N15" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="N16" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="N17" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="N18" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="N19" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="N20" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="N21" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="N23" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="N25" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="N24" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="N26" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="N27" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="N28" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="N30" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="N31" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="N32" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="N34" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="N37" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="N38" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="N39" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="N43" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="N44" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="N6" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="N7" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="N8" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="N9" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="N29" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="N35" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="N36" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="N42" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId39"/>

</xml_diff>